<commit_message>
Update Three Sisters Kitchen demo workbook
Binary update from local Excel testing — not something I authored or
inspected the internal diff of; committing as-is per explicit request.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/demo-data/Three_Sisters_Kitchen_MENTOR_Demo.xlsx
+++ b/src/demo-data/Three_Sisters_Kitchen_MENTOR_Demo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\battu\Mentor\src\demo-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE4381E-229D-434A-9338-FF298A59975E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A7D1170-E939-471A-8807-EC1CC60F9B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README - Ground Truth" sheetId="1" r:id="rId1"/>
@@ -1001,10 +1001,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1184,7 +1180,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="438" row="82">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="7">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>

</xml_diff>